<commit_message>
Actualización automática de resultados
</commit_message>
<xml_diff>
--- a/presidencia/df_validos.xlsx
+++ b/presidencia/df_validos.xlsx
@@ -624,7 +624,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/uc?id=1FEyEnwKzngdyocidRZ4Y2FRZbfGXQcgD</t>
+          <t>https://drive.google.com/uc?id=14hX-tNiuvueC9IXkw8MxYYNa43hDA1DL</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>https://drive.google.com/uc?id=1FEyEnwKzngdyocidRZ4Y2FRZbfGXQcgD</t>
+          <t>https://drive.google.com/uc?id=14hX-tNiuvueC9IXkw8MxYYNa43hDA1DL</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>https://drive.google.com/uc?id=1FEyEnwKzngdyocidRZ4Y2FRZbfGXQcgD</t>
+          <t>https://drive.google.com/uc?id=14hX-tNiuvueC9IXkw8MxYYNa43hDA1DL</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>https://drive.google.com/uc?id=1WTfHZk9AisNxFGwHw8x3y6k5zFSGFzZl</t>
+          <t>https://drive.google.com/uc?id=1f1m1u666bAgWKZZy_SazdB-4mdDux9RH</t>
         </is>
       </c>
     </row>
@@ -1493,7 +1493,7 @@
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>https://drive.google.com/uc?id=1WQ5Qor1_D5Q5ZAE_c-HLrpdUhPIDCOCw</t>
+          <t>https://drive.google.com/uc?id=1f1m1u666bAgWKZZy_SazdB-4mdDux9RH</t>
         </is>
       </c>
     </row>

</xml_diff>